<commit_message>
chore: run 2026-09-07 08:57 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_07_09_2026.xlsx
+++ b/logs/Consolidado_07_09_2026.xlsx
@@ -679,7 +679,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
         <v>4</v>
@@ -698,7 +698,7 @@
         <v>10</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
         <v>9</v>
@@ -4794,12 +4794,12 @@
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>7106530</t>
+          <t>7106534</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
@@ -19777,11 +19777,7 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>8036335</t>
-        </is>
-      </c>
+      <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr">
         <is>
           <t>25%</t>
@@ -19945,12 +19941,12 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>7106530</t>
+          <t>7106534</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>37%</t>
+          <t>40%</t>
         </is>
       </c>
     </row>
@@ -21992,11 +21988,7 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G72" s="3" t="inlineStr">
-        <is>
-          <t>7982207</t>
-        </is>
-      </c>
+      <c r="G72" s="3" t="inlineStr"/>
       <c r="H72" s="3" t="inlineStr">
         <is>
           <t>30%</t>
@@ -30249,11 +30241,7 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>8544717</t>
-        </is>
-      </c>
+      <c r="G34" s="3" t="inlineStr"/>
       <c r="H34" s="3" t="inlineStr">
         <is>
           <t>30%</t>
@@ -31313,11 +31301,7 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>8123760</t>
-        </is>
-      </c>
+      <c r="G60" s="5" t="inlineStr"/>
       <c r="H60" s="5" t="inlineStr">
         <is>
           <t>25%</t>
@@ -40876,7 +40860,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G61" s="5" t="inlineStr"/>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>3066412</t>
+        </is>
+      </c>
       <c r="H61" s="5" t="inlineStr">
         <is>
           <t>25%</t>

</xml_diff>

<commit_message>
chore: run 2026-09-07 21:39 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_07_09_2026.xlsx
+++ b/logs/Consolidado_07_09_2026.xlsx
@@ -752,10 +752,10 @@
         <v>102</v>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E7" t="n">
         <v>6</v>
@@ -790,10 +790,10 @@
         <v>407</v>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E9" t="n">
         <v>3</v>
@@ -7811,37 +7811,37 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="7" t="inlineStr">
+      <c r="A189" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="B189" s="7" t="inlineStr">
+      <c r="B189" s="3" t="inlineStr">
         <is>
           <t>Protetor Solar Réflexe Triasorb SPF50+</t>
         </is>
       </c>
-      <c r="C189" s="7" t="inlineStr">
+      <c r="C189" s="3" t="inlineStr">
         <is>
           <t>30ml</t>
         </is>
       </c>
-      <c r="D189" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E189" s="7" t="inlineStr">
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
         <is>
           <t>428107</t>
         </is>
       </c>
-      <c r="F189" s="7" t="inlineStr">
+      <c r="F189" s="3" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
       </c>
-      <c r="G189" s="7" t="inlineStr">
+      <c r="G189" s="3" t="inlineStr">
         <is>
           <t>https://www.perfumesecompanhia.pt/pt/avene-protetor-solar-reflexe-triasorb-spf50/428107.html</t>
         </is>
@@ -19777,7 +19777,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>8036335</t>
+        </is>
+      </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
           <t>25%</t>
@@ -21988,7 +21992,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G72" s="3" t="inlineStr"/>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>7982207</t>
+        </is>
+      </c>
       <c r="H72" s="3" t="inlineStr">
         <is>
           <t>30%</t>
@@ -30241,7 +30249,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>8544717</t>
+        </is>
+      </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
           <t>30%</t>
@@ -31301,7 +31313,11 @@
           <t>In Stock</t>
         </is>
       </c>
-      <c r="G60" s="5" t="inlineStr"/>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>8123760</t>
+        </is>
+      </c>
       <c r="H60" s="5" t="inlineStr">
         <is>
           <t>25%</t>
@@ -38865,40 +38881,40 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>Elgydium
 Dentrifíco Sensileave Dentes Sensíveis
 50 ml</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>https://wells.pt/dentrifico-sensileave-dentes-sensiveis-7181157.html</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>In Stock</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>Out of Stock</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>7181157</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -44152,47 +44168,47 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>07/09/2026</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>07/09/2026</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>P&amp;C</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Protetor Solar Réflexe Triasorb SPF50+</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>https://www.perfumesecompanhia.pt/pt/avene-protetor-solar-reflexe-triasorb-spf50/428107.html</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>30ml</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>428107</t>
         </is>
       </c>
-      <c r="I23" s="7" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>40%</t>
         </is>
@@ -61699,17 +61715,17 @@
       </c>
       <c r="D397" s="5" t="inlineStr">
         <is>
-          <t>Head Spa Astera Concentrado Refrescante Suavizante</t>
+          <t>Sublime Karité Champô</t>
         </is>
       </c>
       <c r="E397" s="5" t="inlineStr">
         <is>
-          <t>https://www.perfumesecompanhia.pt/pt/rene-furterer-head-spa-astera-concentrado-refrescante-suavizante/428129.html</t>
+          <t>https://www.perfumesecompanhia.pt/pt/rene-furterer-sublime-karite-champo/428132.html</t>
         </is>
       </c>
       <c r="F397" s="5" t="inlineStr">
         <is>
-          <t>50ml</t>
+          <t>200ml</t>
         </is>
       </c>
       <c r="G397" s="6" t="inlineStr">
@@ -61719,12 +61735,12 @@
       </c>
       <c r="H397" s="5" t="inlineStr">
         <is>
-          <t>428129</t>
+          <t>428132</t>
         </is>
       </c>
       <c r="I397" s="5" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -61746,17 +61762,17 @@
       </c>
       <c r="D398" s="3" t="inlineStr">
         <is>
-          <t>Sublime Karité Champô</t>
+          <t>Head Spa Astera Concentrado Refrescante Suavizante</t>
         </is>
       </c>
       <c r="E398" s="3" t="inlineStr">
         <is>
-          <t>https://www.perfumesecompanhia.pt/pt/rene-furterer-sublime-karite-champo/428132.html</t>
+          <t>https://www.perfumesecompanhia.pt/pt/rene-furterer-head-spa-astera-concentrado-refrescante-suavizante/428129.html</t>
         </is>
       </c>
       <c r="F398" s="3" t="inlineStr">
         <is>
-          <t>200ml</t>
+          <t>50ml</t>
         </is>
       </c>
       <c r="G398" s="4" t="inlineStr">
@@ -61766,12 +61782,12 @@
       </c>
       <c r="H398" s="3" t="inlineStr">
         <is>
-          <t>428132</t>
+          <t>428129</t>
         </is>
       </c>
       <c r="I398" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
     </row>

</xml_diff>